<commit_message>
Update couplings database to v2 with 1099.1000+ codes, enlarge photo previews, adjust configurator layout and 3D month badge
</commit_message>
<xml_diff>
--- a/odoo_koppelingen_import_v1.xlsx
+++ b/odoo_koppelingen_import_v1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://interflonbeheer-my.sharepoint.com/personal/kdemeester_interflon_com/Documents/Persoonlijke documenten/Antigravity persoonlijk/Hardware selector/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_30458B4F5712E986385FA871435ED87656CCB5E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E1E7DAE-45E6-4DA9-B643-1B65BFFB2520}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_30458B4F5712E986385FA871435ED87656CCB5E2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8027DD8C-FA0F-4339-81E2-9A2AD45C9170}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1332" uniqueCount="336">
   <si>
     <t>default_code</t>
   </si>
@@ -1028,18 +1028,6 @@
   </si>
   <si>
     <t>Verlengstuk buitendraad 1/4" NPT x binnendraad 1/4" NPT, effectieve lengte 50mm</t>
-  </si>
-  <si>
-    <t>Installatiekit lubricator + single point lubricator</t>
-  </si>
-  <si>
-    <t>Gemengd</t>
-  </si>
-  <si>
-    <t>Hardware / Koppelingen / Installatiekits</t>
-  </si>
-  <si>
-    <t>Installatiekit lubricator + single point lubricator met aansluiting steekkoppeling recht 6mm - G 1/8"</t>
   </si>
 </sst>
 </file>
@@ -1417,7 +1405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5792,40 +5780,6 @@
         <v>335</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A122" s="2"/>
-      <c r="B122" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D122" s="3"/>
-      <c r="E122" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="F122" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G122" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="H122" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I122" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J122" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K122" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="L122" s="3" t="s">
-        <v>339</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>